<commit_message>
[AUTO] Transformación Concrelab - 2026-08-14 20:32:31
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_ALBURA.xlsx
+++ b/DatosTransformados/reporte_concrelab_ALBURA.xlsx
@@ -60939,10 +60939,10 @@
         </is>
       </c>
       <c r="F1345" s="1" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="G1345" s="1" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="H1345" t="n">
         <v>7</v>
@@ -60984,10 +60984,10 @@
         </is>
       </c>
       <c r="F1346" s="1" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="G1346" s="1" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="H1346" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-08-26 12:51:08
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_ALBURA.xlsx
+++ b/DatosTransformados/reporte_concrelab_ALBURA.xlsx
@@ -57335,7 +57335,7 @@
       </c>
       <c r="E1265" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plastico cimentación T4 </t>
+          <t>Vigas Cimentación T4 Ejes 9-12, Placa Ejes 15-13</t>
         </is>
       </c>
       <c r="F1265" s="1" t="n">
@@ -57380,7 +57380,7 @@
       </c>
       <c r="E1266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plastico cimentación T4 </t>
+          <t>Vigas Cimentación T4 Ejes 9-12, Placa Ejes 15-13</t>
         </is>
       </c>
       <c r="F1266" s="1" t="n">
@@ -57425,7 +57425,7 @@
       </c>
       <c r="E1267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plastico cimentación T4 </t>
+          <t>Vigas Cimentación T4 Ejes 9-12, Placa Ejes 15-13</t>
         </is>
       </c>
       <c r="F1267" s="1" t="n">
@@ -57965,7 +57965,7 @@
       </c>
       <c r="E1279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plastico cimentación  T4 </t>
+          <t>Vigas Cimentación T4 Ejes 9-12, Placa Ejes 15-13</t>
         </is>
       </c>
       <c r="F1279" s="1" t="n">
@@ -58010,7 +58010,7 @@
       </c>
       <c r="E1280" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plastico cimentación  T4 </t>
+          <t>Vigas Cimentación T4 Ejes 9-12, Placa Ejes 15-13</t>
         </is>
       </c>
       <c r="F1280" s="1" t="n">
@@ -58055,7 +58055,7 @@
       </c>
       <c r="E1281" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plastico cimentación  T4 </t>
+          <t>Vigas Cimentación T4 Ejes 9-12, Placa Ejes 15-13</t>
         </is>
       </c>
       <c r="F1281" s="1" t="n">

</xml_diff>